<commit_message>
Enhance Arizona tracker with outreach pipeline columns and dropdowns
Add Status, 1st contact date, Channel, Follow-up date, Sample OK?, Sample sent
date, and Tracking # columns with data-validation dropdowns (Status/Channel/
Sample OK?), tinted tracking block, freeze panes, and a README usage sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX28XCL3v6f7LuJT98rxVZ
</commit_message>
<xml_diff>
--- a/07_markets/us/AZ_cafe_outreach.xlsx
+++ b/07_markets/us/AZ_cafe_outreach.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AZ Cafés'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AZ Cafés'!$A$1:$R$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E7EEDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBFAF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -105,6 +110,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -477,26 +485,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
@@ -549,7 +561,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Contacted (date)</t>
+          <t>1st contact (date)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -559,10 +571,30 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Follow-up (date)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Sample OK?</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Sample sent (date)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Tracking #</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Next action</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -612,11 +644,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr"/>
+      <c r="P2" s="4" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -662,11 +706,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr"/>
+      <c r="P3" s="4" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -712,11 +768,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -762,11 +830,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -787,7 +867,7 @@
           <t>Scottsdale</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -812,11 +892,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -837,7 +929,7 @@
           <t>Scottsdale</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -862,11 +954,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -887,7 +991,7 @@
           <t>Scottsdale/Phoenix 多店舗</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -912,11 +1016,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -937,7 +1053,7 @@
           <t>AZ発・多店舗</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -962,11 +1078,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1012,11 +1140,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1062,11 +1202,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1112,11 +1264,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1162,11 +1326,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1212,11 +1388,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1262,11 +1450,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1287,7 +1487,7 @@
           <t>Midtown Phoenix</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1312,11 +1512,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1337,7 +1549,7 @@
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1362,11 +1574,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1387,7 +1611,7 @@
           <t>Downtown Phoenix</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1412,11 +1636,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1437,7 +1673,7 @@
           <t>Central Phoenix</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1462,11 +1698,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1487,7 +1735,7 @@
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1512,11 +1760,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1537,7 +1797,7 @@
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1562,11 +1822,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1587,7 +1859,7 @@
           <t>Downtown Phoenix</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1612,11 +1884,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1637,7 +1921,7 @@
           <t>Tempe(本拠)/多店舗</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1662,11 +1946,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1687,7 +1983,7 @@
           <t>Downtown Chandler</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1712,11 +2008,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1762,11 +2070,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1787,7 +2107,7 @@
           <t>Tempe</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1812,11 +2132,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr"/>
+      <c r="P26" s="4" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1837,7 +2169,7 @@
           <t>Mesa</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1862,11 +2194,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1912,11 +2256,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr"/>
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1962,11 +2318,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2012,11 +2380,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2037,7 +2417,7 @@
           <t>Oak Creek/Sedona</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2062,11 +2442,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2087,7 +2479,7 @@
           <t>Sedona/AZ 多店舗</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2112,11 +2504,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2162,11 +2566,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr"/>
+      <c r="P33" s="4" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2187,7 +2603,7 @@
           <t>Flagstaff</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2212,11 +2628,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr"/>
+      <c r="P34" s="4" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2237,7 +2665,7 @@
           <t>Flagstaff</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2262,11 +2690,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2287,7 +2727,7 @@
           <t>Flagstaff</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2312,11 +2752,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr"/>
+      <c r="P36" s="4" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2337,7 +2789,7 @@
           <t>Flagstaff</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2362,11 +2814,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2412,11 +2876,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr"/>
+      <c r="P38" s="4" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2437,7 +2913,7 @@
           <t>Tucson</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2462,11 +2938,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2487,7 +2975,7 @@
           <t>Tucson</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2512,11 +3000,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr"/>
+      <c r="P40" s="4" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2537,7 +3037,7 @@
           <t>Tucson(Mercado)</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2562,11 +3062,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr"/>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr"/>
+      <c r="P41" s="4" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2587,7 +3099,7 @@
           <t>Tucson</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2612,11 +3124,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr"/>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr"/>
+      <c r="P42" s="4" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2637,7 +3161,7 @@
           <t>Tucson(大学街)</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2662,11 +3186,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
-      <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr"/>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2687,7 +3223,7 @@
           <t>Tucson</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2712,11 +3248,23 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr"/>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="R44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2737,7 +3285,7 @@
           <t>Tucson</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2762,14 +3310,37 @@
           <t>要確認</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
-      <c r="M45" s="2" t="inlineStr"/>
-      <c r="N45" s="2" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr"/>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr"/>
+      <c r="Q45" s="2" t="inlineStr"/>
+      <c r="R45" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:R1"/>
+  <dataValidations count="3">
+    <dataValidation sqref="J2:J45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="状況を選択" type="list">
+      <formula1>"Not started,Contacted,Replied,Sample requested,Sample sent,Negotiating,Won,Lost,No response"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Channel" prompt="連絡チャネルを選択" type="list">
+      <formula1>"Email,IG DM,Website form,Phone,In person,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Sample OK?" prompt="サンプル送付可否" type="list">
+      <formula1>"Pending,Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2780,221 +3351,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="74" customWidth="1" min="2" max="2"/>
+    <col width="86" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>SHIZUNE MATCHA — Arizona Café List</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>SHIZUNE MATCHA — Arizona Café Tracker</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>作成日</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>戦略</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>ハワイの勝ち筋(低飽和×ウェルネス×リゾート×高所得)の再現。Scottsdale(富裕/観光)・Sedona(ウェルネス聖地)を厚めに</t>
-        </is>
-      </c>
+      <c r="A3" s="7" t="inlineStr"/>
+      <c r="B3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="7" t="n"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>列の使い方</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>プルダウン: Not started → Contacted → Replied → Sample requested → Sample sent → Negotiating → Won / Lost / No response</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1st contact (date)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>初回連絡した日（例 2026-10-06）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>プルダウン: Email / IG DM / Website form / Phone / In person / Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Follow-up (date)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>次のフォロー予定日 or 2回目連絡日</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Sample OK?</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>プルダウン: Pending（未定）→ Yes（送付可）/ No（不要）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Sample sent (date)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>サンプルを発送した日（入っていれば＝送付済み）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Tracking #</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>配送追跡番号</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>次にやること（例: 返信待ち・10/12フォロー）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>自由メモ（担当者名・反応など）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>重要</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>実在店を知識ベースで整理。Email/URL/IG・営業状況は送信前に必ず最終確認(サイトContact / wholesale@ / hello@ / Hunter・Apollo)。IGが起点</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Email/URL/IG・営業状況は送信前に要確認。IGが起点→サイトContact / Hunter・Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>A=最優先(抹茶/ウェルネス・観光富裕層フィット) / B=specialtyロースター等 二次</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>物流</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>USD建て・日本直送(FOB/DDU Japan)。送料・関税は買い手負担で明記</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>学び</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>CA=飽和で反応0% / HI=40→4(10%)。AZはHIアナログとして選定</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Region別 件数</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Scottsdale</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Tempe</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Chandler</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Gilbert</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Mesa</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>1</v>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>A=最優先 / B=二次（A=16 / B=28）</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Sedona</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Flagstaff</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Tucson</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr"/>
-      <c r="B21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Tier別</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>A=16 / B=28</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>件数</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>合計 44（Scottsdale 8 / Phoenix 13 / Sedona 5 / Flagstaff 5 / Tucson 8 / 他）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop redundant Sample OK? column from Arizona tracker
Sample interest is already captured by Status = 'Sample requested', so the
separate Sample OK? column is removed. Keeps Sample sent (date) and Tracking #.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX28XCL3v6f7LuJT98rxVZ
</commit_message>
<xml_diff>
--- a/07_markets/us/AZ_cafe_outreach.xlsx
+++ b/07_markets/us/AZ_cafe_outreach.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AZ Cafés'!$A$1:$R$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AZ Cafés'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -501,11 +501,10 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -576,25 +575,20 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Sample OK?</t>
+          <t>Sample sent (date)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Sample sent (date)</t>
+          <t>Tracking #</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Tracking #</t>
+          <t>Next action</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Next action</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -652,15 +646,10 @@
       <c r="K2" s="4" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N2" s="4" t="inlineStr"/>
       <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -714,15 +703,10 @@
       <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N3" s="4" t="inlineStr"/>
       <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -776,15 +760,10 @@
       <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N4" s="4" t="inlineStr"/>
       <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -838,15 +817,10 @@
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N5" s="4" t="inlineStr"/>
       <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -900,15 +874,10 @@
       <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N6" s="4" t="inlineStr"/>
       <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -962,15 +931,10 @@
       <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N7" s="4" t="inlineStr"/>
       <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1024,15 +988,10 @@
       <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N8" s="4" t="inlineStr"/>
       <c r="O8" s="4" t="inlineStr"/>
-      <c r="P8" s="4" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1086,15 +1045,10 @@
       <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1148,15 +1102,10 @@
       <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1210,15 +1159,10 @@
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1272,15 +1216,10 @@
       <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N12" s="4" t="inlineStr"/>
       <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1334,15 +1273,10 @@
       <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1396,15 +1330,10 @@
       <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1458,15 +1387,10 @@
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1520,15 +1444,10 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1582,15 +1501,10 @@
       <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1644,15 +1558,10 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1706,15 +1615,10 @@
       <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N19" s="4" t="inlineStr"/>
       <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1768,15 +1672,10 @@
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1830,15 +1729,10 @@
       <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N21" s="4" t="inlineStr"/>
       <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1892,15 +1786,10 @@
       <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N22" s="4" t="inlineStr"/>
       <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1954,15 +1843,10 @@
       <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N23" s="4" t="inlineStr"/>
       <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2016,15 +1900,10 @@
       <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N24" s="4" t="inlineStr"/>
       <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2078,15 +1957,10 @@
       <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N25" s="4" t="inlineStr"/>
       <c r="O25" s="4" t="inlineStr"/>
-      <c r="P25" s="4" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2140,15 +2014,10 @@
       <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N26" s="4" t="inlineStr"/>
       <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2202,15 +2071,10 @@
       <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N27" s="4" t="inlineStr"/>
       <c r="O27" s="4" t="inlineStr"/>
-      <c r="P27" s="4" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2264,15 +2128,10 @@
       <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N28" s="4" t="inlineStr"/>
       <c r="O28" s="4" t="inlineStr"/>
-      <c r="P28" s="4" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2326,15 +2185,10 @@
       <c r="K29" s="4" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N29" s="4" t="inlineStr"/>
       <c r="O29" s="4" t="inlineStr"/>
-      <c r="P29" s="4" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2388,15 +2242,10 @@
       <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N30" s="4" t="inlineStr"/>
       <c r="O30" s="4" t="inlineStr"/>
-      <c r="P30" s="4" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2450,15 +2299,10 @@
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
       <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N31" s="4" t="inlineStr"/>
       <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2512,15 +2356,10 @@
       <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="4" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N32" s="4" t="inlineStr"/>
       <c r="O32" s="4" t="inlineStr"/>
-      <c r="P32" s="4" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
       <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2574,15 +2413,10 @@
       <c r="K33" s="4" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="4" t="inlineStr"/>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N33" s="4" t="inlineStr"/>
       <c r="O33" s="4" t="inlineStr"/>
-      <c r="P33" s="4" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
       <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2636,15 +2470,10 @@
       <c r="K34" s="4" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N34" s="4" t="inlineStr"/>
       <c r="O34" s="4" t="inlineStr"/>
-      <c r="P34" s="4" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2698,15 +2527,10 @@
       <c r="K35" s="4" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N35" s="4" t="inlineStr"/>
       <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr"/>
       <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2760,15 +2584,10 @@
       <c r="K36" s="4" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N36" s="4" t="inlineStr"/>
       <c r="O36" s="4" t="inlineStr"/>
-      <c r="P36" s="4" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
       <c r="Q36" s="2" t="inlineStr"/>
-      <c r="R36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2822,15 +2641,10 @@
       <c r="K37" s="4" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N37" s="4" t="inlineStr"/>
       <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
       <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2884,15 +2698,10 @@
       <c r="K38" s="4" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N38" s="4" t="inlineStr"/>
       <c r="O38" s="4" t="inlineStr"/>
-      <c r="P38" s="4" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
-      <c r="R38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2946,15 +2755,10 @@
       <c r="K39" s="4" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N39" s="4" t="inlineStr"/>
       <c r="O39" s="4" t="inlineStr"/>
-      <c r="P39" s="4" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
       <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3008,15 +2812,10 @@
       <c r="K40" s="4" t="inlineStr"/>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N40" s="4" t="inlineStr"/>
       <c r="O40" s="4" t="inlineStr"/>
-      <c r="P40" s="4" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3070,15 +2869,10 @@
       <c r="K41" s="4" t="inlineStr"/>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N41" s="4" t="inlineStr"/>
       <c r="O41" s="4" t="inlineStr"/>
-      <c r="P41" s="4" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
       <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3132,15 +2926,10 @@
       <c r="K42" s="4" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr"/>
       <c r="M42" s="4" t="inlineStr"/>
-      <c r="N42" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N42" s="4" t="inlineStr"/>
       <c r="O42" s="4" t="inlineStr"/>
-      <c r="P42" s="4" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr"/>
       <c r="Q42" s="2" t="inlineStr"/>
-      <c r="R42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3194,15 +2983,10 @@
       <c r="K43" s="4" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr"/>
       <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N43" s="4" t="inlineStr"/>
       <c r="O43" s="4" t="inlineStr"/>
-      <c r="P43" s="4" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
       <c r="Q43" s="2" t="inlineStr"/>
-      <c r="R43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3256,15 +3040,10 @@
       <c r="K44" s="4" t="inlineStr"/>
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr"/>
-      <c r="N44" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N44" s="4" t="inlineStr"/>
       <c r="O44" s="4" t="inlineStr"/>
-      <c r="P44" s="4" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
       <c r="Q44" s="2" t="inlineStr"/>
-      <c r="R44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3318,27 +3097,19 @@
       <c r="K45" s="4" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr"/>
       <c r="M45" s="4" t="inlineStr"/>
-      <c r="N45" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="N45" s="4" t="inlineStr"/>
       <c r="O45" s="4" t="inlineStr"/>
-      <c r="P45" s="4" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr"/>
       <c r="Q45" s="2" t="inlineStr"/>
-      <c r="R45" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:Q1"/>
+  <dataValidations count="2">
     <dataValidation sqref="J2:J45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="状況を選択" type="list">
       <formula1>"Not started,Contacted,Replied,Sample requested,Sample sent,Negotiating,Won,Lost,No response"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Channel" prompt="連絡チャネルを選択" type="list">
       <formula1>"Email,IG DM,Website form,Phone,In person,Other"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Sample OK?" prompt="サンプル送付可否" type="list">
-      <formula1>"Pending,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3440,66 +3211,66 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Sample OK?</t>
+          <t>Sample sent (date)</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>プルダウン: Pending（未定）→ Yes（送付可）/ No（不要）</t>
+          <t>サンプルを発送した日（入っていれば＝送付済み）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Sample sent (date)</t>
+          <t>Tracking #</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>サンプルを発送した日（入っていれば＝送付済み）</t>
+          <t>配送追跡番号</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Tracking #</t>
+          <t>Next action</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>配送追跡番号</t>
+          <t>次にやること（例: 返信待ち・10/12フォロー）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Next action</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>次にやること（例: 返信待ち・10/12フォロー）</t>
+          <t>自由メモ（担当者名・反応など）</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>自由メモ（担当者名・反応など）</t>
-        </is>
-      </c>
+      <c r="A13" s="7" t="inlineStr"/>
+      <c r="B13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-      <c r="B14" s="8" t="n"/>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>補足</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>「サンプル希望」はStatusの Sample requested で表現（専用列は廃止）</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">

</xml_diff>